<commit_message>
Update Healthmap data and analysis scripts
Replaced Healthmap data file with 'HealthmapData.csv' and updated all references in R and Python scripts. Adjusted date ranges for analysis and visualizations to start from January 1, 2023. Enhanced data aggregation and plotting logic in fig1.R, fig2.R, and fig4.R, including new summary tables and improved figure layouts. Added new data files and removed outdated ones to reflect the latest dataset.
</commit_message>
<xml_diff>
--- a/Outcome/fig data/fig 4.xlsx
+++ b/Outcome/fig data/fig 4.xlsx
@@ -1,63 +1,80 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="false"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://6kmwxn-my.sharepoint.com/personal/kanggle_globalinfectiousdisease_com/Documents/XMU/likangguo/2024/06 pertussis/PertussisIncidence/Outcome/fig data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="9" documentId="11_22D5943C40872B1923C39D1A5E0949434AF4E6DB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA2FB5ED-5924-4DBF-8683-06B464F1EF3F}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$C$72</definedName>
+  </definedNames>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="11">
   <si>
-    <t xml:space="preserve">country</t>
+    <t>country</t>
   </si>
   <si>
-    <t xml:space="preserve">Year</t>
+    <t>Year</t>
   </si>
   <si>
-    <t xml:space="preserve">MedianAge</t>
+    <t>MedianAge</t>
   </si>
   <si>
-    <t xml:space="preserve">AU</t>
+    <t>AU</t>
   </si>
   <si>
-    <t xml:space="preserve">CN</t>
+    <t>CN</t>
   </si>
   <si>
-    <t xml:space="preserve">GB</t>
+    <t>GB</t>
   </si>
   <si>
-    <t xml:space="preserve">JP</t>
+    <t>JP</t>
   </si>
   <si>
-    <t xml:space="preserve">NZ</t>
+    <t>NZ</t>
   </si>
   <si>
-    <t xml:space="preserve">SE</t>
+    <t>SE</t>
   </si>
   <si>
-    <t xml:space="preserve">SG</t>
+    <t>SG</t>
   </si>
   <si>
-    <t xml:space="preserve">US</t>
+    <t>US</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -85,9 +102,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -369,11 +395,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C72"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -384,789 +410,791 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2">
         <v>2015</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>15.9</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3">
         <v>2016</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3">
         <v>15.4</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4">
         <v>2017</v>
       </c>
-      <c r="C4" t="n">
-        <v>17.9</v>
-      </c>
-    </row>
-    <row r="5">
+      <c r="C4">
+        <v>17.899999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B5">
         <v>2018</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5">
         <v>14.8</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>3</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B6">
         <v>2019</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6">
         <v>15.4</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>3</v>
       </c>
-      <c r="B7" t="n">
+      <c r="B7">
         <v>2020</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7">
         <v>23.6</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>3</v>
       </c>
-      <c r="B8" t="n">
+      <c r="B8">
         <v>2021</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8">
         <v>38.6</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>3</v>
       </c>
-      <c r="B9" t="n">
+      <c r="B9">
         <v>2022</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9">
         <v>41.9</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>3</v>
       </c>
-      <c r="B10" t="n">
+      <c r="B10">
         <v>2023</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10">
         <v>15</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>3</v>
       </c>
-      <c r="B11" t="n">
+      <c r="B11">
         <v>2024</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11">
         <v>13.1</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>4</v>
       </c>
-      <c r="B12" t="n">
+      <c r="B12">
         <v>2015</v>
       </c>
-      <c r="C12" t="n">
-        <v>2.3</v>
-      </c>
-    </row>
-    <row r="13">
+      <c r="C12">
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>4</v>
       </c>
-      <c r="B13" t="n">
+      <c r="B13">
         <v>2016</v>
       </c>
-      <c r="C13" t="n">
-        <v>2.3</v>
-      </c>
-    </row>
-    <row r="14">
+      <c r="C13">
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>4</v>
       </c>
-      <c r="B14" t="n">
+      <c r="B14">
         <v>2017</v>
       </c>
-      <c r="C14" t="n">
-        <v>2.3</v>
-      </c>
-    </row>
-    <row r="15">
+      <c r="C14">
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>4</v>
       </c>
-      <c r="B15" t="n">
+      <c r="B15">
         <v>2018</v>
       </c>
-      <c r="C15" t="n">
-        <v>2.3</v>
-      </c>
-    </row>
-    <row r="16">
+      <c r="C15">
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>4</v>
       </c>
-      <c r="B16" t="n">
+      <c r="B16">
         <v>2019</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16">
         <v>2.4</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>4</v>
       </c>
-      <c r="B17" t="n">
+      <c r="B17">
         <v>2020</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17">
         <v>2.5</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>4</v>
       </c>
-      <c r="B18" t="n">
+      <c r="B18">
         <v>2021</v>
       </c>
-      <c r="C18" t="n">
+      <c r="C18">
         <v>3.5</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>4</v>
       </c>
-      <c r="B19" t="n">
+      <c r="B19">
         <v>2022</v>
       </c>
-      <c r="C19" t="n">
+      <c r="C19">
         <v>3.9</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>4</v>
       </c>
-      <c r="B20" t="n">
+      <c r="B20">
         <v>2023</v>
       </c>
-      <c r="C20" t="n">
+      <c r="C20">
         <v>3.7</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>5</v>
       </c>
-      <c r="B21" t="n">
+      <c r="B21">
         <v>2015</v>
       </c>
-      <c r="C21" t="n">
+      <c r="C21">
         <v>27.1</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>5</v>
       </c>
-      <c r="B22" t="n">
+      <c r="B22">
         <v>2016</v>
       </c>
-      <c r="C22" t="n">
+      <c r="C22">
         <v>31.7</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>5</v>
       </c>
-      <c r="B23" t="n">
+      <c r="B23">
         <v>2017</v>
       </c>
-      <c r="C23" t="n">
+      <c r="C23">
         <v>31.1</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>5</v>
       </c>
-      <c r="B24" t="n">
+      <c r="B24">
         <v>2018</v>
       </c>
-      <c r="C24" t="n">
+      <c r="C24">
         <v>32.5</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>5</v>
       </c>
-      <c r="B25" t="n">
+      <c r="B25">
         <v>2019</v>
       </c>
-      <c r="C25" t="n">
+      <c r="C25">
         <v>29.8</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>5</v>
       </c>
-      <c r="B26" t="n">
+      <c r="B26">
         <v>2020</v>
       </c>
-      <c r="C26" t="n">
+      <c r="C26">
         <v>43.4</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>5</v>
       </c>
-      <c r="B27" t="n">
+      <c r="B27">
         <v>2021</v>
       </c>
-      <c r="C27" t="n">
+      <c r="C27">
         <v>46.1</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>5</v>
       </c>
-      <c r="B28" t="n">
+      <c r="B28">
         <v>2022</v>
       </c>
-      <c r="C28" t="n">
+      <c r="C28">
         <v>36.5</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>5</v>
       </c>
-      <c r="B29" t="n">
+      <c r="B29">
         <v>2023</v>
       </c>
-      <c r="C29" t="n">
-        <v>18.4</v>
-      </c>
-    </row>
-    <row r="30">
+      <c r="C29">
+        <v>18.399999999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>5</v>
       </c>
-      <c r="B30" t="n">
+      <c r="B30">
         <v>2024</v>
       </c>
-      <c r="C30" t="n">
+      <c r="C30">
         <v>27.6</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>6</v>
       </c>
-      <c r="B31" t="n">
+      <c r="B31">
         <v>2018</v>
       </c>
-      <c r="C31" t="n">
+      <c r="C31">
         <v>11.2</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>6</v>
       </c>
-      <c r="B32" t="n">
+      <c r="B32">
         <v>2019</v>
       </c>
-      <c r="C32" t="n">
+      <c r="C32">
         <v>11.4</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>6</v>
       </c>
-      <c r="B33" t="n">
+      <c r="B33">
         <v>2020</v>
       </c>
-      <c r="C33" t="n">
+      <c r="C33">
         <v>12.6</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>6</v>
       </c>
-      <c r="B34" t="n">
+      <c r="B34">
         <v>2021</v>
       </c>
-      <c r="C34" t="n">
+      <c r="C34">
         <v>13.2</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>6</v>
       </c>
-      <c r="B35" t="n">
+      <c r="B35">
         <v>2022</v>
       </c>
-      <c r="C35" t="n">
+      <c r="C35">
         <v>13.3</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>6</v>
       </c>
-      <c r="B36" t="n">
+      <c r="B36">
         <v>2023</v>
       </c>
-      <c r="C36" t="n">
+      <c r="C36">
         <v>10.4</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>7</v>
       </c>
-      <c r="B37" t="n">
+      <c r="B37">
         <v>2015</v>
       </c>
-      <c r="C37" t="n">
+      <c r="C37">
         <v>22.9</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>7</v>
       </c>
-      <c r="B38" t="n">
+      <c r="B38">
         <v>2016</v>
       </c>
-      <c r="C38" t="n">
+      <c r="C38">
         <v>25.1</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>7</v>
       </c>
-      <c r="B39" t="n">
+      <c r="B39">
         <v>2017</v>
       </c>
-      <c r="C39" t="n">
+      <c r="C39">
         <v>19</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>7</v>
       </c>
-      <c r="B40" t="n">
+      <c r="B40">
         <v>2018</v>
       </c>
-      <c r="C40" t="n">
+      <c r="C40">
         <v>20.6</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>7</v>
       </c>
-      <c r="B41" t="n">
+      <c r="B41">
         <v>2019</v>
       </c>
-      <c r="C41" t="n">
+      <c r="C41">
         <v>25.9</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>7</v>
       </c>
-      <c r="B42" t="n">
+      <c r="B42">
         <v>2020</v>
       </c>
-      <c r="C42" t="n">
+      <c r="C42">
         <v>21.1</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>7</v>
       </c>
-      <c r="B43" t="n">
+      <c r="B43">
         <v>2021</v>
       </c>
-      <c r="C43" t="n">
-        <v>37.2</v>
-      </c>
-    </row>
-    <row r="44">
+      <c r="C43">
+        <v>37.200000000000003</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>7</v>
       </c>
-      <c r="B44" t="n">
+      <c r="B44">
         <v>2022</v>
       </c>
-      <c r="C44" t="n">
+      <c r="C44">
         <v>32.4</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>7</v>
       </c>
-      <c r="B45" t="n">
+      <c r="B45">
         <v>2023</v>
       </c>
-      <c r="C45" t="n">
+      <c r="C45">
         <v>10.9</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>7</v>
       </c>
-      <c r="B46" t="n">
+      <c r="B46">
         <v>2024</v>
       </c>
-      <c r="C46" t="n">
+      <c r="C46">
         <v>13.6</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>8</v>
       </c>
-      <c r="B47" t="n">
+      <c r="B47">
         <v>2015</v>
       </c>
-      <c r="C47" t="n">
+      <c r="C47">
         <v>23.5</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>8</v>
       </c>
-      <c r="B48" t="n">
+      <c r="B48">
         <v>2016</v>
       </c>
-      <c r="C48" t="n">
+      <c r="C48">
         <v>22.9</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>8</v>
       </c>
-      <c r="B49" t="n">
+      <c r="B49">
         <v>2017</v>
       </c>
-      <c r="C49" t="n">
+      <c r="C49">
         <v>25.9</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>8</v>
       </c>
-      <c r="B50" t="n">
+      <c r="B50">
         <v>2018</v>
       </c>
-      <c r="C50" t="n">
+      <c r="C50">
         <v>26.1</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>8</v>
       </c>
-      <c r="B51" t="n">
+      <c r="B51">
         <v>2019</v>
       </c>
-      <c r="C51" t="n">
+      <c r="C51">
         <v>28.1</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>8</v>
       </c>
-      <c r="B52" t="n">
+      <c r="B52">
         <v>2020</v>
       </c>
-      <c r="C52" t="n">
+      <c r="C52">
         <v>21.7</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>8</v>
       </c>
-      <c r="B53" t="n">
+      <c r="B53">
         <v>2021</v>
       </c>
-      <c r="C53" t="n">
+      <c r="C53">
         <v>40.6</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>8</v>
       </c>
-      <c r="B54" t="n">
+      <c r="B54">
         <v>2022</v>
       </c>
-      <c r="C54" t="n">
+      <c r="C54">
         <v>31.2</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>8</v>
       </c>
-      <c r="B55" t="n">
+      <c r="B55">
         <v>2023</v>
       </c>
-      <c r="C55" t="n">
+      <c r="C55">
         <v>23.1</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>8</v>
       </c>
-      <c r="B56" t="n">
+      <c r="B56">
         <v>2024</v>
       </c>
-      <c r="C56" t="n">
+      <c r="C56">
         <v>28</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>9</v>
       </c>
-      <c r="B57" t="n">
+      <c r="B57">
         <v>2015</v>
       </c>
-      <c r="C57" t="n">
+      <c r="C57">
         <v>3.3</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>9</v>
       </c>
-      <c r="B58" t="n">
+      <c r="B58">
         <v>2016</v>
       </c>
-      <c r="C58" t="n">
+      <c r="C58">
         <v>6.1</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>9</v>
       </c>
-      <c r="B59" t="n">
+      <c r="B59">
         <v>2017</v>
       </c>
-      <c r="C59" t="n">
+      <c r="C59">
         <v>6.7</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>9</v>
       </c>
-      <c r="B60" t="n">
+      <c r="B60">
         <v>2018</v>
       </c>
-      <c r="C60" t="n">
+      <c r="C60">
         <v>7.1</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>9</v>
       </c>
-      <c r="B61" t="n">
+      <c r="B61">
         <v>2019</v>
       </c>
-      <c r="C61" t="n">
+      <c r="C61">
         <v>7.9</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>9</v>
       </c>
-      <c r="B62" t="n">
+      <c r="B62">
         <v>2020</v>
       </c>
-      <c r="C62" t="n">
+      <c r="C62">
         <v>57.9</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>10</v>
       </c>
-      <c r="B63" t="n">
+      <c r="B63">
         <v>2015</v>
       </c>
-      <c r="C63" t="n">
+      <c r="C63">
         <v>11.6</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>10</v>
       </c>
-      <c r="B64" t="n">
+      <c r="B64">
         <v>2016</v>
       </c>
-      <c r="C64" t="n">
+      <c r="C64">
         <v>12.3</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>10</v>
       </c>
-      <c r="B65" t="n">
+      <c r="B65">
         <v>2017</v>
       </c>
-      <c r="C65" t="n">
+      <c r="C65">
         <v>11.9</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>10</v>
       </c>
-      <c r="B66" t="n">
+      <c r="B66">
         <v>2018</v>
       </c>
-      <c r="C66" t="n">
+      <c r="C66">
         <v>11.4</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>10</v>
       </c>
-      <c r="B67" t="n">
+      <c r="B67">
         <v>2019</v>
       </c>
-      <c r="C67" t="n">
+      <c r="C67">
         <v>11.7</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>10</v>
       </c>
-      <c r="B68" t="n">
+      <c r="B68">
         <v>2020</v>
       </c>
-      <c r="C68" t="n">
+      <c r="C68">
         <v>12</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>10</v>
       </c>
-      <c r="B69" t="n">
+      <c r="B69">
         <v>2021</v>
       </c>
-      <c r="C69" t="n">
+      <c r="C69">
         <v>29</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>10</v>
       </c>
-      <c r="B70" t="n">
+      <c r="B70">
         <v>2022</v>
       </c>
-      <c r="C70" t="n">
+      <c r="C70">
         <v>14.5</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>10</v>
       </c>
-      <c r="B71" t="n">
+      <c r="B71">
         <v>2023</v>
       </c>
-      <c r="C71" t="n">
-        <v>8.7</v>
-      </c>
-    </row>
-    <row r="72">
+      <c r="C71">
+        <v>8.6999999999999993</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>10</v>
       </c>
-      <c r="B72" t="n">
+      <c r="B72">
         <v>2024</v>
       </c>
-      <c r="C72" t="n">
+      <c r="C72">
         <v>12.4</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C72" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>